<commit_message>
Adds historical vintage subranges, finishes early industrial equipment retirement implementation, pending cleanup
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
+++ b/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\ctrl-settings\MV\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\ctrl-settings\MV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5EA5CF-754F-487E-818D-4C1FCEBCB68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CFDC8DF-4CD0-4EA0-96A7-695A7F473FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="-27660" yWindow="270" windowWidth="27270" windowHeight="16395" activeTab="5" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="MV-current" sheetId="3" r:id="rId3"/>
     <sheet name="MV-preceding" sheetId="4" r:id="rId4"/>
     <sheet name="FMV" sheetId="5" r:id="rId5"/>
+    <sheet name="MV-historical" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="264">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -3907,4 +3908,374 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AA3F29F-5B20-495C-833F-1BC19D331C2C}">
+  <dimension ref="A1:A72"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>229</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Integrates clean industrial heat PTC into cash flows
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
+++ b/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\ctrl-settings\MV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CFDC8DF-4CD0-4EA0-96A7-695A7F473FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07520257-4DF5-470B-B226-1D68A8C3DB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27660" yWindow="270" windowWidth="27270" windowHeight="16395" activeTab="5" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="-25890" yWindow="1080" windowWidth="21600" windowHeight="12645" activeTab="6" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="MV-preceding" sheetId="4" r:id="rId4"/>
     <sheet name="FMV" sheetId="5" r:id="rId5"/>
     <sheet name="MV-historical" sheetId="6" r:id="rId6"/>
+    <sheet name="MV-run" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="264">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -4278,4 +4279,169 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0A6D85D-6D7E-4F19-8E78-99221E312E4F}">
+  <dimension ref="A1:A31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Correct historical vintages file to include all historical years
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
+++ b/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ctrl-settings\MV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97893DB4-850B-4BC0-AA77-26C3A9AB5EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099C2261-0F08-4DBE-A5AB-FBCD78181648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="222">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -523,6 +523,183 @@
   </si>
   <si>
     <t>include all vintages except the final year.</t>
+  </si>
+  <si>
+    <t>Vintage1891</t>
+  </si>
+  <si>
+    <t>Vintage1892</t>
+  </si>
+  <si>
+    <t>Vintage1893</t>
+  </si>
+  <si>
+    <t>Vintage1894</t>
+  </si>
+  <si>
+    <t>Vintage1895</t>
+  </si>
+  <si>
+    <t>Vintage1896</t>
+  </si>
+  <si>
+    <t>Vintage1897</t>
+  </si>
+  <si>
+    <t>Vintage1898</t>
+  </si>
+  <si>
+    <t>Vintage1899</t>
+  </si>
+  <si>
+    <t>Vintage1900</t>
+  </si>
+  <si>
+    <t>Vintage1901</t>
+  </si>
+  <si>
+    <t>Vintage1902</t>
+  </si>
+  <si>
+    <t>Vintage1903</t>
+  </si>
+  <si>
+    <t>Vintage1904</t>
+  </si>
+  <si>
+    <t>Vintage1905</t>
+  </si>
+  <si>
+    <t>Vintage1906</t>
+  </si>
+  <si>
+    <t>Vintage1907</t>
+  </si>
+  <si>
+    <t>Vintage1908</t>
+  </si>
+  <si>
+    <t>Vintage1909</t>
+  </si>
+  <si>
+    <t>Vintage1910</t>
+  </si>
+  <si>
+    <t>Vintage1911</t>
+  </si>
+  <si>
+    <t>Vintage1912</t>
+  </si>
+  <si>
+    <t>Vintage1913</t>
+  </si>
+  <si>
+    <t>Vintage1914</t>
+  </si>
+  <si>
+    <t>Vintage1915</t>
+  </si>
+  <si>
+    <t>Vintage1916</t>
+  </si>
+  <si>
+    <t>Vintage1917</t>
+  </si>
+  <si>
+    <t>Vintage1918</t>
+  </si>
+  <si>
+    <t>Vintage1919</t>
+  </si>
+  <si>
+    <t>Vintage1920</t>
+  </si>
+  <si>
+    <t>Vintage1921</t>
+  </si>
+  <si>
+    <t>Vintage1922</t>
+  </si>
+  <si>
+    <t>Vintage1923</t>
+  </si>
+  <si>
+    <t>Vintage1924</t>
+  </si>
+  <si>
+    <t>Vintage1925</t>
+  </si>
+  <si>
+    <t>Vintage1926</t>
+  </si>
+  <si>
+    <t>Vintage1927</t>
+  </si>
+  <si>
+    <t>Vintage1928</t>
+  </si>
+  <si>
+    <t>Vintage1929</t>
+  </si>
+  <si>
+    <t>Vintage1930</t>
+  </si>
+  <si>
+    <t>Vintage1931</t>
+  </si>
+  <si>
+    <t>Vintage1932</t>
+  </si>
+  <si>
+    <t>Vintage1933</t>
+  </si>
+  <si>
+    <t>Vintage1934</t>
+  </si>
+  <si>
+    <t>Vintage1935</t>
+  </si>
+  <si>
+    <t>Vintage1936</t>
+  </si>
+  <si>
+    <t>Vintage1937</t>
+  </si>
+  <si>
+    <t>Vintage1938</t>
+  </si>
+  <si>
+    <t>Vintage1939</t>
+  </si>
+  <si>
+    <t>Vintage1940</t>
+  </si>
+  <si>
+    <t>Vintage1941</t>
+  </si>
+  <si>
+    <t>Vintage1942</t>
+  </si>
+  <si>
+    <t>Vintage1943</t>
+  </si>
+  <si>
+    <t>Vintage1944</t>
+  </si>
+  <si>
+    <t>Vintage1945</t>
+  </si>
+  <si>
+    <t>Vintage1946</t>
+  </si>
+  <si>
+    <t>Vintage1947</t>
+  </si>
+  <si>
+    <t>Vintage1948</t>
+  </si>
+  <si>
+    <t>Vintage1949</t>
   </si>
 </sst>
 </file>
@@ -572,9 +749,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -889,7 +1069,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1D3264-BEAA-43D0-A5CC-06C5D3B72BE0}">
-  <dimension ref="A1:B166"/>
+  <dimension ref="A1:B225"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -944,757 +1124,1052 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A84" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A104" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A105" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A107" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A108" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A109" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A110" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A111" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A112" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A113" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A114" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A115" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A116" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A117" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A118" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A119" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A120" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A121" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A122" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A123" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A124" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A125" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A126" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A127" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A128" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A129" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A130" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A131" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A132" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A133" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A134" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A135" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A136" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A137" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A138" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A139" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A140" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A141" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A142" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A143" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A144" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A145" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A146" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A147" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A148" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A149" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A150" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A151" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A152" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A153" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A154" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A155" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A156" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A157" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A158" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A159" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A160" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A161" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A103" t="s">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A162" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A163" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A164" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A106" t="s">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A165" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A107" t="s">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A166" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A108" t="s">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A167" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A109" t="s">
+    <row r="168" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A168" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A110" t="s">
+    <row r="169" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A169" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A111" t="s">
+    <row r="170" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A170" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A112" t="s">
+    <row r="171" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A171" s="2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A113" t="s">
+    <row r="172" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A172" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A114" t="s">
+    <row r="173" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A173" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A115" t="s">
+    <row r="174" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A174" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A116" t="s">
+    <row r="175" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A175" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A117" t="s">
+    <row r="176" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A176" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A118" t="s">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A177" s="2" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A119" t="s">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A178" s="2" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A120" t="s">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A179" s="2" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A121" t="s">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A180" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A122" t="s">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A181" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A123" t="s">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A182" s="2" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A124" t="s">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A183" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A125" t="s">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A184" s="2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A126" t="s">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A185" s="2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A127" t="s">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A186" s="2" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A128" t="s">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A187" s="2" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A129" t="s">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A188" s="2" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A130" t="s">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A189" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A131" t="s">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A190" s="2" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A132" t="s">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A191" s="2" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A133" t="s">
+    <row r="192" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A192" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A134" t="s">
+    <row r="193" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A193" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A135" t="s">
+    <row r="194" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A194" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A136" t="s">
+    <row r="195" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A195" s="2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A137" t="s">
+    <row r="196" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A196" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A138" t="s">
+    <row r="197" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A197" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A139" t="s">
+    <row r="198" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A198" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A140" t="s">
+    <row r="199" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A199" s="2" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A141" t="s">
+    <row r="200" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A200" s="2" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A142" t="s">
+    <row r="201" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A201" s="2" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A143" t="s">
+    <row r="202" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A202" s="2" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A144" t="s">
+    <row r="203" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A203" s="2" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A145" t="s">
+    <row r="204" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A204" s="2" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A146" t="s">
+    <row r="205" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A205" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A147" t="s">
+    <row r="206" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A206" s="2" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A148" t="s">
+    <row r="207" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A207" s="2" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A149" t="s">
+    <row r="208" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A208" s="2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A150" t="s">
+    <row r="209" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A209" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A151" t="s">
+    <row r="210" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A210" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A152" t="s">
+    <row r="211" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A211" s="2" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A153" t="s">
+    <row r="212" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A212" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A154" t="s">
+    <row r="213" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A213" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A155" t="s">
+    <row r="214" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A214" s="2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A156" t="s">
+    <row r="215" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A215" s="2" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A157" t="s">
+    <row r="216" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A216" s="2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A158" t="s">
+    <row r="217" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A217" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A159" t="s">
+    <row r="218" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A218" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A160" t="s">
+    <row r="219" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A219" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A161" t="s">
+    <row r="220" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A220" s="2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A162" t="s">
+    <row r="221" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A221" s="2" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A163" t="s">
+    <row r="222" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A222" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A164" t="s">
+    <row r="223" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A223" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A165" t="s">
+    <row r="224" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A224" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A166" t="s">
+    <row r="225" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A225" s="2" t="s">
         <v>157</v>
       </c>
     </row>
@@ -1709,8 +2184,11 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:A72"/>
+  <dimension ref="A1:A131"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1718,429 +2196,653 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" t="str">
-        <f>About!A16</f>
-        <v>Vintage1950</v>
+      <c r="A2" s="2" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" t="str">
-        <f>About!A17</f>
-        <v>Vintage1951</v>
+      <c r="A3" s="2" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" t="str">
-        <f>About!A18</f>
-        <v>Vintage1952</v>
+      <c r="A4" s="2" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" t="str">
-        <f>About!A19</f>
-        <v>Vintage1953</v>
+      <c r="A5" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" t="str">
-        <f>About!A20</f>
-        <v>Vintage1954</v>
+      <c r="A6" s="2" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" t="str">
-        <f>About!A21</f>
-        <v>Vintage1955</v>
+      <c r="A7" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" t="str">
-        <f>About!A22</f>
-        <v>Vintage1956</v>
+      <c r="A8" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" t="str">
-        <f>About!A23</f>
-        <v>Vintage1957</v>
+      <c r="A9" s="2" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" t="str">
-        <f>About!A24</f>
-        <v>Vintage1958</v>
+      <c r="A10" s="2" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" t="str">
-        <f>About!A25</f>
-        <v>Vintage1959</v>
+      <c r="A11" s="2" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" t="str">
-        <f>About!A26</f>
-        <v>Vintage1960</v>
+      <c r="A12" s="2" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" t="str">
-        <f>About!A27</f>
-        <v>Vintage1961</v>
+      <c r="A13" s="2" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" t="str">
-        <f>About!A28</f>
-        <v>Vintage1962</v>
+      <c r="A14" s="2" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" t="str">
-        <f>About!A29</f>
-        <v>Vintage1963</v>
+      <c r="A15" s="2" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" t="str">
-        <f>About!A30</f>
-        <v>Vintage1964</v>
+      <c r="A16" s="2" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="str">
-        <f>About!A31</f>
-        <v>Vintage1965</v>
+      <c r="A17" s="2" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" t="str">
-        <f>About!A32</f>
-        <v>Vintage1966</v>
+      <c r="A18" s="2" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" t="str">
-        <f>About!A33</f>
-        <v>Vintage1967</v>
+      <c r="A19" s="2" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" t="str">
-        <f>About!A34</f>
-        <v>Vintage1968</v>
+      <c r="A20" s="2" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" t="str">
-        <f>About!A35</f>
-        <v>Vintage1969</v>
+      <c r="A21" s="2" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="str">
-        <f>About!A36</f>
-        <v>Vintage1970</v>
+      <c r="A22" s="2" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="str">
-        <f>About!A37</f>
-        <v>Vintage1971</v>
+      <c r="A23" s="2" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="str">
-        <f>About!A38</f>
-        <v>Vintage1972</v>
+      <c r="A24" s="2" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="str">
-        <f>About!A39</f>
-        <v>Vintage1973</v>
+      <c r="A25" s="2" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="str">
-        <f>About!A40</f>
-        <v>Vintage1974</v>
+      <c r="A26" s="2" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="str">
-        <f>About!A41</f>
-        <v>Vintage1975</v>
+      <c r="A27" s="2" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="str">
-        <f>About!A42</f>
-        <v>Vintage1976</v>
+      <c r="A28" s="2" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="str">
-        <f>About!A43</f>
-        <v>Vintage1977</v>
+      <c r="A29" s="2" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="str">
-        <f>About!A44</f>
-        <v>Vintage1978</v>
+      <c r="A30" s="2" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="str">
-        <f>About!A45</f>
-        <v>Vintage1979</v>
+      <c r="A31" s="2" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="str">
-        <f>About!A46</f>
-        <v>Vintage1980</v>
+      <c r="A32" s="2" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="str">
-        <f>About!A47</f>
-        <v>Vintage1981</v>
+      <c r="A33" s="2" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="str">
-        <f>About!A48</f>
-        <v>Vintage1982</v>
+      <c r="A34" s="2" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="str">
-        <f>About!A49</f>
-        <v>Vintage1983</v>
+      <c r="A35" s="2" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="str">
-        <f>About!A50</f>
-        <v>Vintage1984</v>
+      <c r="A36" s="2" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="str">
-        <f>About!A51</f>
-        <v>Vintage1985</v>
+      <c r="A37" s="2" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="str">
-        <f>About!A52</f>
-        <v>Vintage1986</v>
+      <c r="A38" s="2" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="str">
-        <f>About!A53</f>
-        <v>Vintage1987</v>
+      <c r="A39" s="2" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="str">
-        <f>About!A54</f>
-        <v>Vintage1988</v>
+      <c r="A40" s="2" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" t="str">
-        <f>About!A55</f>
-        <v>Vintage1989</v>
+      <c r="A41" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="str">
-        <f>About!A56</f>
-        <v>Vintage1990</v>
+      <c r="A42" s="2" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" t="str">
-        <f>About!A57</f>
-        <v>Vintage1991</v>
+      <c r="A43" s="2" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="str">
-        <f>About!A58</f>
-        <v>Vintage1992</v>
+      <c r="A44" s="2" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="str">
-        <f>About!A59</f>
-        <v>Vintage1993</v>
+      <c r="A45" s="2" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="str">
-        <f>About!A60</f>
-        <v>Vintage1994</v>
+      <c r="A46" s="2" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" t="str">
-        <f>About!A61</f>
-        <v>Vintage1995</v>
+      <c r="A47" s="2" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" t="str">
-        <f>About!A62</f>
-        <v>Vintage1996</v>
+      <c r="A48" s="2" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="str">
-        <f>About!A63</f>
-        <v>Vintage1997</v>
+      <c r="A49" s="2" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="str">
-        <f>About!A64</f>
-        <v>Vintage1998</v>
+      <c r="A50" s="2" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" t="str">
-        <f>About!A65</f>
-        <v>Vintage1999</v>
+      <c r="A51" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" t="str">
-        <f>About!A66</f>
-        <v>Vintage2000</v>
+      <c r="A52" s="2" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" t="str">
-        <f>About!A67</f>
-        <v>Vintage2001</v>
+      <c r="A53" s="2" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" t="str">
-        <f>About!A68</f>
-        <v>Vintage2002</v>
+      <c r="A54" s="2" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" t="str">
-        <f>About!A69</f>
-        <v>Vintage2003</v>
+      <c r="A55" s="2" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" t="str">
-        <f>About!A70</f>
-        <v>Vintage2004</v>
+      <c r="A56" s="2" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" t="str">
-        <f>About!A71</f>
-        <v>Vintage2005</v>
+      <c r="A57" s="2" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" t="str">
-        <f>About!A72</f>
-        <v>Vintage2006</v>
+      <c r="A58" s="2" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" t="str">
-        <f>About!A73</f>
-        <v>Vintage2007</v>
+      <c r="A59" s="2" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A60" t="str">
-        <f>About!A74</f>
-        <v>Vintage2008</v>
+      <c r="A60" s="2" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A61" t="str">
-        <f>About!A75</f>
-        <v>Vintage2009</v>
+      <c r="A61" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A62" t="str">
-        <f>About!A76</f>
-        <v>Vintage2010</v>
+      <c r="A62" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A63" t="str">
-        <f>About!A77</f>
-        <v>Vintage2011</v>
+      <c r="A63" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A64" t="str">
-        <f>About!A78</f>
-        <v>Vintage2012</v>
+      <c r="A64" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A65" t="str">
-        <f>About!A79</f>
-        <v>Vintage2013</v>
+      <c r="A65" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A66" t="str">
-        <f>About!A80</f>
-        <v>Vintage2014</v>
+      <c r="A66" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" t="str">
-        <f>About!A81</f>
-        <v>Vintage2015</v>
+      <c r="A67" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A68" t="str">
-        <f>About!A82</f>
-        <v>Vintage2016</v>
+      <c r="A68" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A69" t="str">
-        <f>About!A83</f>
-        <v>Vintage2017</v>
+      <c r="A69" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A70" t="str">
-        <f>About!A84</f>
-        <v>Vintage2018</v>
+      <c r="A70" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A71" t="str">
-        <f>About!A85</f>
-        <v>Vintage2019</v>
+      <c r="A71" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A72" t="str">
-        <f>About!A86</f>
-        <v>Vintage2020</v>
+      <c r="A72" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A84" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A104" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A105" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A107" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A108" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A109" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A110" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A111" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A112" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A113" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A114" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A115" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A116" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A117" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A118" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A119" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A120" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A121" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A122" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A123" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A124" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A125" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A126" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A127" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A128" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A129" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A130" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A131" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update start year files to reference 2023 data and set the initial time to 2024 in Vensim
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
+++ b/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ctrl-settings\MV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099C2261-0F08-4DBE-A5AB-FBCD78181648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D35DF3F-8EA7-4636-902F-2FFDDC0E0CB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="222">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -2184,7 +2184,7 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:A131"/>
+  <dimension ref="A1:A134"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.54296875" customWidth="1"/>
@@ -2845,6 +2845,21 @@
         <v>77</v>
       </c>
     </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A132" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A133" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A134" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Adjusts start year in MV
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
+++ b/InputData/ctrl-settings/MV/Modeled Vintages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ctrl-settings\MV\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\ctrl-settings\MV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D35DF3F-8EA7-4636-902F-2FFDDC0E0CB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A8B2B3-39E0-4579-9C19-3EA6F04EF46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="-27675" yWindow="1485" windowWidth="24795" windowHeight="15195" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="222">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -1070,14 +1070,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1D3264-BEAA-43D0-A5CC-06C5D3B72BE0}">
   <dimension ref="A1:B225"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1085,7 +1085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1093,1082 +1093,1082 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="203" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="205" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="206" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="207" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="208" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="210" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="211" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="212" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="213" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="214" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="215" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="216" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="217" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="218" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="219" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="220" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="221" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="222" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="223" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="224" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="225" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
         <v>157</v>
       </c>
@@ -2184,680 +2184,685 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:A134"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A135"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" s="2" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>